<commit_message>
informacion publica segundo trimestre 2023
</commit_message>
<xml_diff>
--- a/assets/archivos/TRANSPARENCIA/ART 63 COMUNES 2023/2DO_TRIMESTRE/FRACC 64/LTAIPT_A64F01IG1.xlsx
+++ b/assets/archivos/TRANSPARENCIA/ART 63 COMUNES 2023/2DO_TRIMESTRE/FRACC 64/LTAIPT_A64F01IG1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="330" yWindow="495" windowWidth="19815" windowHeight="9405"/>
+    <workbookView xWindow="330" yWindow="555" windowWidth="19815" windowHeight="8385"/>
   </bookViews>
   <sheets>
     <sheet name="Informacion" sheetId="1" r:id="rId1"/>
@@ -139,31 +139,31 @@
     <t>Nota</t>
   </si>
   <si>
-    <t>2022</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
-    <t>EEB39E7F0E5604E8F41726B76C524EC2</t>
-  </si>
-  <si>
-    <t>01/04/2022</t>
-  </si>
-  <si>
-    <t>30/06/2022</t>
-  </si>
-  <si>
-    <t>08/05/2022</t>
-  </si>
-  <si>
-    <t>Transparencia y Archivo</t>
-  </si>
-  <si>
-    <t>11/07/2022</t>
-  </si>
-  <si>
-    <t>Del periodo del 01 de abril del 2021 al 30 de junio del 2021, el Colegio de Bachilleres del Estado de Tlaxcala, Con fundamento en el artìculo 4 y 73, fracciòn XVI Bases 2a y 3a de la Carta Magna;  El Colegio de Bachilleres del Estado de Tlaxcala, devido al ACUERDO por el que se establecen las medidas preventivas que se deberán implementar para la mitigación y control de los riesgos para la salud que implica la enfermedad por el virus SARS-CoV2 (COVID-19). En virtud de lo anterior el Subsistema no cuenta por el momento con dictámenes de Iniciativas de carácter legal vinculadas con sus atribuciones.</t>
+    <t>Área de Transparencia</t>
+  </si>
+  <si>
+    <t>2023</t>
+  </si>
+  <si>
+    <t>1183CA9DF44A54CE0968A5341E935537</t>
+  </si>
+  <si>
+    <t>01/04/2023</t>
+  </si>
+  <si>
+    <t>06/06/2023</t>
+  </si>
+  <si>
+    <t>15/04/2023</t>
+  </si>
+  <si>
+    <t>10/07/2023</t>
+  </si>
+  <si>
+    <t>Durante el periodo del 01 de abril de 2023 al 30 de junio del 2023, el Colegio de Bachilleres del Estado de Tlaxcala no cuenta por el momento con Dictámenes de Iniciativas de carácter legal, vinculadas con sus atribuciones.</t>
   </si>
 </sst>
 </file>
@@ -559,7 +559,7 @@
   <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.5703125" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="36" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="38.5703125" bestFit="1" customWidth="1"/>
@@ -766,40 +766,40 @@
     </row>
     <row r="8" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L8" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>48</v>

</xml_diff>